<commit_message>
Add PM2 config, frontend server & model delete
Add PM2 ecosystem and frontend start files, a simple Express frontend server, and PM2 npm scripts; add start-frontend helper. Implement permanent model deletion flow: add deletePermanente API call in frontend service and admin-only delete UI + confirmation dialog in ModelosPage. Enhance export pipeline: rebuild exportarPlantillaMaestra to produce a 189-column template (headers, column numbers) and map EquipamientoModelo columns into ordered rows for Excel. Improve equipamiento handling: safer OtrosDatos JSON parsing, record FechaCreacion on create and avoid inserting it dynamically. Add db utility querySequentialOnSingleConn for running multiple queries on one connection. Also add/update sample/brand Excel files and other small adjustments.
</commit_message>
<xml_diff>
--- a/data/muestra Plantilla_Maestra_Autos_Completa.xlsx
+++ b/data/muestra Plantilla_Maestra_Autos_Completa.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Autodata\Autodata\Temporales Autodata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\servidor2024\Temporales Autodata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{273F57E4-D026-4338-B433-38CF62C555C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8CB6EA3-90EF-40FF-B7F1-0AB4FFDF62C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{48D503FB-514F-4C9A-9E6A-D4966E14396E}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1637" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1650" uniqueCount="361">
   <si>
     <t>Marca</t>
   </si>
@@ -1090,6 +1090,36 @@
   </si>
   <si>
     <t>estas columnas estan en nuestra base original y no en la que generaste vos.</t>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>Tipo Motor</t>
+  </si>
+  <si>
+    <t>Tipo Caja Automática</t>
+  </si>
+  <si>
+    <t>Tipo</t>
+  </si>
+  <si>
+    <t>Importador</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>convertidor de par</t>
+  </si>
+  <si>
+    <t>AUTOMOVIL</t>
+  </si>
+  <si>
+    <t>SANTA ROSA AUTOMOTORES</t>
+  </si>
+  <si>
+    <t>Convertidor de par</t>
   </si>
 </sst>
 </file>
@@ -1197,7 +1227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1213,6 +1243,9 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1552,1130 +1585,1154 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:GC12"/>
+  <dimension ref="A1:GG12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="59.19921875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:185" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:189" x14ac:dyDescent="0.3">
+      <c r="A1" s="11">
+        <v>1</v>
+      </c>
+      <c r="B1" s="11">
+        <v>2</v>
+      </c>
+      <c r="C1" s="11">
+        <v>3</v>
+      </c>
+      <c r="D1" s="11">
+        <v>4</v>
+      </c>
+      <c r="E1" s="11">
+        <v>5</v>
+      </c>
+      <c r="F1" s="11">
+        <v>6</v>
+      </c>
+      <c r="G1" s="11">
+        <v>7</v>
+      </c>
+      <c r="H1" s="11">
+        <v>8</v>
+      </c>
+      <c r="I1" s="11">
+        <v>9</v>
+      </c>
+      <c r="J1" s="11">
+        <v>10</v>
+      </c>
+      <c r="K1" s="11">
+        <v>11</v>
+      </c>
+      <c r="L1" s="11">
+        <v>12</v>
+      </c>
+      <c r="M1" s="11">
+        <v>13</v>
+      </c>
+      <c r="N1" s="11">
+        <v>14</v>
+      </c>
+      <c r="O1" s="11">
+        <v>15</v>
+      </c>
+      <c r="P1" s="11">
+        <v>16</v>
+      </c>
+      <c r="Q1" s="11">
+        <v>17</v>
+      </c>
+      <c r="R1" s="11">
+        <v>18</v>
+      </c>
+      <c r="S1" s="11">
+        <v>19</v>
+      </c>
+      <c r="T1" s="11">
+        <v>20</v>
+      </c>
+      <c r="U1" s="11">
+        <v>21</v>
+      </c>
+      <c r="V1" s="11">
+        <v>22</v>
+      </c>
+      <c r="W1" s="11">
+        <v>23</v>
+      </c>
+      <c r="X1" s="11">
+        <v>24</v>
+      </c>
+      <c r="Y1" s="11">
+        <v>25</v>
+      </c>
+      <c r="Z1" s="11">
+        <v>26</v>
+      </c>
+      <c r="AA1" s="11">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="11">
+        <v>28</v>
+      </c>
+      <c r="AC1" s="11">
+        <v>29</v>
+      </c>
+      <c r="AD1" s="11">
+        <v>30</v>
+      </c>
+      <c r="AE1" s="11">
+        <v>31</v>
+      </c>
+      <c r="AF1" s="11">
+        <v>32</v>
+      </c>
+      <c r="AG1" s="11">
+        <v>33</v>
+      </c>
+      <c r="AH1" s="11">
+        <v>34</v>
+      </c>
+      <c r="AI1" s="11">
+        <v>35</v>
+      </c>
+      <c r="AJ1" s="11">
+        <v>36</v>
+      </c>
+      <c r="AK1" s="11">
+        <v>37</v>
+      </c>
+      <c r="AL1" s="11">
+        <v>38</v>
+      </c>
+      <c r="AM1" s="11">
+        <v>39</v>
+      </c>
+      <c r="AN1" s="11">
+        <v>40</v>
+      </c>
+      <c r="AO1" s="11">
+        <v>41</v>
+      </c>
+      <c r="AP1" s="11">
+        <v>42</v>
+      </c>
+      <c r="AQ1" s="11">
+        <v>43</v>
+      </c>
+      <c r="AR1" s="11">
+        <v>44</v>
+      </c>
+      <c r="AS1" s="11">
+        <v>45</v>
+      </c>
+      <c r="AT1" s="11">
+        <v>46</v>
+      </c>
+      <c r="AU1" s="11">
+        <v>47</v>
+      </c>
+      <c r="AV1" s="11">
+        <v>48</v>
+      </c>
+      <c r="AW1" s="11">
+        <v>49</v>
+      </c>
+      <c r="AX1" s="11">
+        <v>50</v>
+      </c>
+      <c r="AY1" s="11">
+        <v>51</v>
+      </c>
+      <c r="AZ1" s="11">
+        <v>52</v>
+      </c>
+      <c r="BA1" s="11">
+        <v>53</v>
+      </c>
+      <c r="BB1" s="11">
+        <v>54</v>
+      </c>
+      <c r="BC1" s="11">
+        <v>55</v>
+      </c>
+      <c r="BD1" s="11">
+        <v>56</v>
+      </c>
+      <c r="BE1" s="11">
+        <v>57</v>
+      </c>
+      <c r="BF1" s="11">
+        <v>58</v>
+      </c>
+      <c r="BG1" s="11">
+        <v>59</v>
+      </c>
+      <c r="BH1" s="11">
+        <v>60</v>
+      </c>
+      <c r="BI1" s="11">
+        <v>61</v>
+      </c>
+      <c r="BJ1" s="11">
+        <v>62</v>
+      </c>
+      <c r="BK1" s="11">
+        <v>63</v>
+      </c>
+      <c r="BL1" s="11">
+        <v>64</v>
+      </c>
+      <c r="BM1" s="11">
+        <v>65</v>
+      </c>
+      <c r="BN1" s="11">
+        <v>66</v>
+      </c>
+      <c r="BO1" s="11">
+        <v>67</v>
+      </c>
+      <c r="BP1" s="11">
+        <v>68</v>
+      </c>
+      <c r="BQ1" s="11">
+        <v>69</v>
+      </c>
+      <c r="BR1" s="11">
+        <v>70</v>
+      </c>
+      <c r="BS1" s="11">
+        <v>71</v>
+      </c>
+      <c r="BT1" s="11">
+        <v>72</v>
+      </c>
+      <c r="BU1" s="11">
+        <v>73</v>
+      </c>
+      <c r="BV1" s="11">
+        <v>74</v>
+      </c>
+      <c r="BW1" s="11">
+        <v>75</v>
+      </c>
+      <c r="BX1" s="11">
+        <v>76</v>
+      </c>
+      <c r="BY1" s="11">
+        <v>77</v>
+      </c>
+      <c r="BZ1" s="11">
+        <v>78</v>
+      </c>
+      <c r="CA1" s="11">
+        <v>79</v>
+      </c>
+      <c r="CB1" s="11">
+        <v>80</v>
+      </c>
+      <c r="CC1" s="11">
+        <v>81</v>
+      </c>
+      <c r="CD1" s="11">
+        <v>82</v>
+      </c>
+      <c r="CE1" s="11">
+        <v>83</v>
+      </c>
+      <c r="CF1" s="11">
+        <v>84</v>
+      </c>
+      <c r="CG1" s="11">
+        <v>85</v>
+      </c>
+      <c r="CH1" s="11">
+        <v>86</v>
+      </c>
+      <c r="CI1" s="11">
+        <v>87</v>
+      </c>
+      <c r="CJ1" s="11">
+        <v>88</v>
+      </c>
+      <c r="CK1" s="11">
+        <v>89</v>
+      </c>
+      <c r="CL1" s="11">
+        <v>90</v>
+      </c>
+      <c r="CM1" s="11">
+        <v>91</v>
+      </c>
+      <c r="CN1" s="11">
+        <v>92</v>
+      </c>
+      <c r="CO1" s="11">
+        <v>93</v>
+      </c>
+      <c r="CP1" s="11">
+        <v>94</v>
+      </c>
+      <c r="CQ1" s="11">
+        <v>95</v>
+      </c>
+      <c r="CR1" s="11">
+        <v>96</v>
+      </c>
+      <c r="CS1" s="11">
+        <v>97</v>
+      </c>
+      <c r="CT1" s="11">
+        <v>98</v>
+      </c>
+      <c r="CU1" s="11">
+        <v>99</v>
+      </c>
+      <c r="CV1" s="11">
+        <v>100</v>
+      </c>
+      <c r="CW1" s="11">
+        <v>101</v>
+      </c>
+      <c r="CX1" s="11">
+        <v>102</v>
+      </c>
+      <c r="CY1" s="11">
+        <v>103</v>
+      </c>
+      <c r="CZ1" s="11">
+        <v>104</v>
+      </c>
+      <c r="DA1" s="11">
+        <v>105</v>
+      </c>
+      <c r="DB1" s="11">
+        <v>106</v>
+      </c>
+      <c r="DC1" s="11">
+        <v>107</v>
+      </c>
+      <c r="DD1" s="11">
+        <v>108</v>
+      </c>
+      <c r="DE1" s="11">
+        <v>109</v>
+      </c>
+      <c r="DF1" s="11">
+        <v>110</v>
+      </c>
+      <c r="DG1" s="11">
+        <v>111</v>
+      </c>
+      <c r="DH1" s="11">
+        <v>112</v>
+      </c>
+      <c r="DI1" s="11">
+        <v>113</v>
+      </c>
+      <c r="DJ1" s="11">
+        <v>114</v>
+      </c>
+      <c r="DK1" s="11">
+        <v>115</v>
+      </c>
+      <c r="DL1" s="11">
+        <v>116</v>
+      </c>
+      <c r="DM1" s="11">
+        <v>117</v>
+      </c>
+      <c r="DN1" s="11">
+        <v>118</v>
+      </c>
+      <c r="DO1" s="11">
+        <v>119</v>
+      </c>
+      <c r="DP1" s="11">
+        <v>120</v>
+      </c>
+      <c r="DQ1" s="11">
+        <v>121</v>
+      </c>
+      <c r="DR1" s="11">
+        <v>122</v>
+      </c>
+      <c r="DS1" s="11">
+        <v>123</v>
+      </c>
+      <c r="DT1" s="11">
+        <v>124</v>
+      </c>
+      <c r="DU1" s="11">
+        <v>125</v>
+      </c>
+      <c r="DV1" s="11">
+        <v>126</v>
+      </c>
+      <c r="DW1" s="11">
+        <v>127</v>
+      </c>
+      <c r="DX1" s="11">
+        <v>128</v>
+      </c>
+      <c r="DY1" s="11">
+        <v>129</v>
+      </c>
+      <c r="DZ1" s="11">
+        <v>130</v>
+      </c>
+      <c r="EA1" s="11">
+        <v>131</v>
+      </c>
+      <c r="EB1" s="11">
+        <v>132</v>
+      </c>
+      <c r="EC1" s="11">
+        <v>133</v>
+      </c>
+      <c r="ED1" s="11">
+        <v>134</v>
+      </c>
+      <c r="EE1" s="11">
+        <v>135</v>
+      </c>
+      <c r="EF1" s="11">
+        <v>136</v>
+      </c>
+      <c r="EG1" s="11">
+        <v>137</v>
+      </c>
+      <c r="EH1" s="11">
+        <v>138</v>
+      </c>
+      <c r="EI1" s="11">
+        <v>139</v>
+      </c>
+      <c r="EJ1" s="11">
+        <v>140</v>
+      </c>
+      <c r="EK1" s="11">
+        <v>141</v>
+      </c>
+      <c r="EL1" s="11">
+        <v>142</v>
+      </c>
+      <c r="EM1" s="11">
+        <v>143</v>
+      </c>
+      <c r="EN1" s="11">
+        <v>144</v>
+      </c>
+      <c r="EO1" s="11">
+        <v>145</v>
+      </c>
+      <c r="EP1" s="11">
+        <v>146</v>
+      </c>
+      <c r="EQ1" s="11">
+        <v>147</v>
+      </c>
+      <c r="ER1" s="11">
+        <v>148</v>
+      </c>
+      <c r="ES1" s="11">
+        <v>149</v>
+      </c>
+      <c r="ET1" s="11">
+        <v>150</v>
+      </c>
+      <c r="EU1" s="11">
+        <v>151</v>
+      </c>
+      <c r="EV1" s="11">
+        <v>152</v>
+      </c>
+      <c r="EW1" s="11">
+        <v>153</v>
+      </c>
+      <c r="EX1" s="11">
+        <v>154</v>
+      </c>
+      <c r="EY1" s="11">
+        <v>155</v>
+      </c>
+      <c r="EZ1" s="11">
+        <v>156</v>
+      </c>
+      <c r="FA1" s="11">
+        <v>157</v>
+      </c>
+      <c r="FB1" s="11">
+        <v>158</v>
+      </c>
+      <c r="FC1" s="11">
+        <v>159</v>
+      </c>
+      <c r="FD1" s="11">
+        <v>160</v>
+      </c>
+      <c r="FE1" s="11">
+        <v>161</v>
+      </c>
+      <c r="FF1" s="11">
+        <v>162</v>
+      </c>
+      <c r="FG1" s="11">
+        <v>163</v>
+      </c>
+      <c r="FH1" s="11">
+        <v>164</v>
+      </c>
+      <c r="FI1" s="11">
+        <v>165</v>
+      </c>
+      <c r="FJ1" s="11">
+        <v>166</v>
+      </c>
+      <c r="FK1" s="11">
+        <v>167</v>
+      </c>
+      <c r="FL1" s="11">
+        <v>168</v>
+      </c>
+      <c r="FM1" s="11">
+        <v>169</v>
+      </c>
+      <c r="FN1" s="11">
+        <v>170</v>
+      </c>
+      <c r="FO1" s="11">
+        <v>171</v>
+      </c>
+      <c r="FP1" s="11">
+        <v>172</v>
+      </c>
+      <c r="FQ1" s="11">
+        <v>173</v>
+      </c>
+      <c r="FR1" s="11">
+        <v>174</v>
+      </c>
+      <c r="FS1" s="11">
+        <v>175</v>
+      </c>
+      <c r="FT1" s="11">
+        <v>176</v>
+      </c>
+      <c r="FU1" s="11">
+        <v>177</v>
+      </c>
+      <c r="FV1" s="11">
+        <v>178</v>
+      </c>
+      <c r="FW1" s="11">
+        <v>179</v>
+      </c>
+      <c r="FX1" s="11">
+        <v>180</v>
+      </c>
+      <c r="FY1" s="11">
+        <v>181</v>
+      </c>
+      <c r="FZ1" s="11">
+        <v>182</v>
+      </c>
+      <c r="GA1" s="11">
+        <v>183</v>
+      </c>
+      <c r="GB1" s="11">
+        <v>184</v>
+      </c>
+      <c r="GC1" s="11">
+        <v>185</v>
+      </c>
+      <c r="GD1" s="11">
+        <v>186</v>
+      </c>
+      <c r="GE1" s="11">
+        <v>187</v>
+      </c>
+      <c r="GF1" s="11">
+        <v>188</v>
+      </c>
+      <c r="GG1" s="11">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="2" spans="1:189" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Y2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="4" t="s">
+      <c r="Z2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="4" t="s">
+      <c r="AA2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="4" t="s">
+      <c r="AB2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="4" t="s">
+      <c r="AC2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" s="4" t="s">
+      <c r="AD2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="4" t="s">
+      <c r="AE2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" s="4" t="s">
+      <c r="AF2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" s="4" t="s">
+      <c r="AG2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" s="4" t="s">
+      <c r="AH2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" s="4" t="s">
+      <c r="AI2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" s="4" t="s">
+      <c r="AJ2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="AK1" s="4" t="s">
+      <c r="AK2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="AL1" s="4" t="s">
+      <c r="AL2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AM1" s="4" t="s">
+      <c r="AM2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="AN1" s="4" t="s">
+      <c r="AN2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AO1" s="4" t="s">
+      <c r="AO2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AP1" s="4" t="s">
+      <c r="AP2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="AQ1" s="4" t="s">
+      <c r="AQ2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AR1" s="4" t="s">
+      <c r="AR2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AS1" s="4" t="s">
+      <c r="AS2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AT1" s="4" t="s">
+      <c r="AT2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="AU1" s="4" t="s">
+      <c r="AU2" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AV1" s="4" t="s">
+      <c r="AV2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="AW1" s="4" t="s">
+      <c r="AW2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AX1" s="4" t="s">
+      <c r="AX2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="AY1" s="4" t="s">
+      <c r="AY2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AZ1" s="4" t="s">
+      <c r="AZ2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="BA1" s="4" t="s">
+      <c r="BA2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="BB1" s="4" t="s">
+      <c r="BB2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="BC1" s="4" t="s">
+      <c r="BC2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="BD1" s="4" t="s">
+      <c r="BD2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="BE1" s="4" t="s">
+      <c r="BE2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="BF1" s="4" t="s">
+      <c r="BF2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="BG1" s="4" t="s">
+      <c r="BG2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="BH1" s="4" t="s">
+      <c r="BH2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="BI1" s="4" t="s">
+      <c r="BI2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="BJ1" s="4" t="s">
+      <c r="BJ2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="BK1" s="4" t="s">
+      <c r="BK2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="BL1" s="4" t="s">
+      <c r="BL2" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="BM1" s="4" t="s">
+      <c r="BM2" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="BN1" s="4" t="s">
+      <c r="BN2" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="BO1" s="4" t="s">
+      <c r="BO2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="BP1" s="4" t="s">
+      <c r="BP2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="BQ1" s="4" t="s">
+      <c r="BQ2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="BR1" s="4" t="s">
+      <c r="BR2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="BS1" s="4" t="s">
+      <c r="BS2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="BT1" s="4" t="s">
+      <c r="BT2" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="BU1" s="4" t="s">
+      <c r="BU2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="BV1" s="4" t="s">
+      <c r="BV2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="BW1" s="4" t="s">
+      <c r="BW2" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="BX1" s="4" t="s">
+      <c r="BX2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="BY1" s="4" t="s">
+      <c r="BY2" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="BZ1" s="4" t="s">
+      <c r="BZ2" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="CA1" s="4" t="s">
+      <c r="CA2" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="CB1" s="4" t="s">
+      <c r="CB2" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="CC1" s="4" t="s">
+      <c r="CC2" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="CD1" s="4" t="s">
+      <c r="CD2" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="CE1" s="4" t="s">
+      <c r="CE2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="CF1" s="4" t="s">
+      <c r="CF2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="CG1" s="4" t="s">
+      <c r="CG2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="CH1" s="4" t="s">
+      <c r="CH2" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="CI1" s="4" t="s">
+      <c r="CI2" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="CJ1" s="4" t="s">
+      <c r="CJ2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="CK1" s="4" t="s">
+      <c r="CK2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="CL1" s="4" t="s">
+      <c r="CL2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="CM1" s="4" t="s">
+      <c r="CM2" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="CN1" s="4" t="s">
+      <c r="CN2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="CO1" s="4" t="s">
+      <c r="CO2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="CP1" s="4" t="s">
+      <c r="CP2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="CQ1" s="4" t="s">
+      <c r="CQ2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="CR1" s="4" t="s">
+      <c r="CR2" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="CS1" s="4" t="s">
+      <c r="CS2" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="CT1" s="4" t="s">
+      <c r="CT2" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="CU1" s="4" t="s">
+      <c r="CU2" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="CV1" s="4" t="s">
+      <c r="CV2" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="CW1" s="4" t="s">
+      <c r="CW2" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="CX1" s="4" t="s">
+      <c r="CX2" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="CY1" s="4" t="s">
+      <c r="CY2" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="CZ1" s="4" t="s">
+      <c r="CZ2" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="DA1" s="4" t="s">
+      <c r="DA2" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="DB1" s="4" t="s">
+      <c r="DB2" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="DC1" s="4" t="s">
+      <c r="DC2" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="DD1" s="4" t="s">
+      <c r="DD2" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="DE1" s="4" t="s">
+      <c r="DE2" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="DF1" s="4" t="s">
+      <c r="DF2" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="DG1" s="4" t="s">
+      <c r="DG2" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="DH1" s="4" t="s">
+      <c r="DH2" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="DI1" s="4" t="s">
+      <c r="DI2" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="DJ1" s="4" t="s">
+      <c r="DJ2" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="DK1" s="4" t="s">
+      <c r="DK2" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="DL1" s="4" t="s">
+      <c r="DL2" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="DM1" s="4" t="s">
+      <c r="DM2" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="DN1" s="4" t="s">
+      <c r="DN2" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="DO1" s="4" t="s">
+      <c r="DO2" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="DP1" s="4" t="s">
+      <c r="DP2" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="DQ1" s="4" t="s">
+      <c r="DQ2" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="DR1" s="4" t="s">
+      <c r="DR2" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="DS1" s="4" t="s">
+      <c r="DS2" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="DT1" s="4" t="s">
+      <c r="DT2" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="DU1" s="4" t="s">
+      <c r="DU2" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="DV1" s="4" t="s">
+      <c r="DV2" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="DW1" s="4" t="s">
+      <c r="DW2" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="DX1" s="4" t="s">
+      <c r="DX2" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="DY1" s="4" t="s">
+      <c r="DY2" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="DZ1" s="4" t="s">
+      <c r="DZ2" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="EA1" s="4" t="s">
+      <c r="EA2" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="EB1" s="4" t="s">
+      <c r="EB2" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="EC1" s="4" t="s">
+      <c r="EC2" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="ED1" s="4" t="s">
+      <c r="ED2" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="EE1" s="4" t="s">
+      <c r="EE2" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="EF1" s="4" t="s">
+      <c r="EF2" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="EG1" s="4" t="s">
+      <c r="EG2" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="EH1" s="4" t="s">
+      <c r="EH2" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="EI1" s="4" t="s">
+      <c r="EI2" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="EJ1" s="4" t="s">
+      <c r="EJ2" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="EK1" s="4" t="s">
+      <c r="EK2" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="EL1" s="4" t="s">
+      <c r="EL2" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="EM1" s="4" t="s">
+      <c r="EM2" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="EN1" s="4" t="s">
+      <c r="EN2" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="EO1" s="4" t="s">
+      <c r="EO2" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="EP1" s="4" t="s">
+      <c r="EP2" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="EQ1" s="4" t="s">
+      <c r="EQ2" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="ER1" s="4" t="s">
+      <c r="ER2" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="ES1" s="4" t="s">
+      <c r="ES2" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="ET1" s="4" t="s">
+      <c r="ET2" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="EU1" s="4" t="s">
+      <c r="EU2" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="EV1" s="4" t="s">
+      <c r="EV2" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="EW1" s="4" t="s">
+      <c r="EW2" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="EX1" s="4" t="s">
+      <c r="EX2" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="EY1" s="4" t="s">
+      <c r="EY2" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="EZ1" s="4" t="s">
+      <c r="EZ2" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="FA1" s="4" t="s">
+      <c r="FA2" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="FB1" s="4" t="s">
+      <c r="FB2" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="FC1" s="4" t="s">
+      <c r="FC2" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="FD1" s="4" t="s">
+      <c r="FD2" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="FE1" s="4" t="s">
+      <c r="FE2" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="FF1" s="4" t="s">
+      <c r="FF2" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="FG1" s="4" t="s">
+      <c r="FG2" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="FH1" s="4" t="s">
+      <c r="FH2" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="FI1" s="4" t="s">
+      <c r="FI2" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="FJ1" s="4" t="s">
+      <c r="FJ2" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="FK1" s="4" t="s">
+      <c r="FK2" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="FL1" s="4" t="s">
+      <c r="FL2" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="FM1" s="4" t="s">
+      <c r="FM2" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="FN1" s="4" t="s">
+      <c r="FN2" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="FO1" s="4" t="s">
+      <c r="FO2" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="FP1" s="4" t="s">
+      <c r="FP2" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="FQ1" s="4" t="s">
+      <c r="FQ2" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="FR1" s="4" t="s">
+      <c r="FR2" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="FS1" s="4" t="s">
+      <c r="FS2" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="FT1" s="4" t="s">
+      <c r="FT2" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="FU1" s="4" t="s">
+      <c r="FU2" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="FV1" s="4" t="s">
+      <c r="FV2" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="FW1" s="4" t="s">
+      <c r="FW2" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="FX1" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="FY1" s="4" t="s">
+      <c r="FX2" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="FZ1" s="4" t="s">
+      <c r="FY2" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="GA1" s="4" t="s">
+      <c r="FZ2" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="GB1" s="4" t="s">
+      <c r="GA2" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="GC1" s="4" t="s">
+      <c r="GB2" s="4" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="2" spans="1:185" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="GC2" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="GD2" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="GE2" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="GF2" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="GG2" s="4" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="3" spans="1:189" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>292</v>
-      </c>
-      <c r="B2" t="s">
-        <v>291</v>
-      </c>
-      <c r="C2" t="s">
-        <v>345</v>
-      </c>
-      <c r="D2" t="s">
-        <v>346</v>
-      </c>
-      <c r="E2" t="s">
-        <v>299</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="G2" t="s">
-        <v>304</v>
-      </c>
-      <c r="H2" t="s">
-        <v>300</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>4335</v>
-      </c>
-      <c r="K2">
-        <v>1825</v>
-      </c>
-      <c r="L2">
-        <v>1660</v>
-      </c>
-      <c r="M2">
-        <v>2600</v>
-      </c>
-      <c r="N2">
-        <v>1390</v>
-      </c>
-      <c r="O2">
-        <v>12.086956521739131</v>
-      </c>
-      <c r="P2" t="s">
-        <v>305</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>283</v>
-      </c>
-      <c r="R2">
-        <v>17</v>
-      </c>
-      <c r="S2" t="s">
-        <v>283</v>
-      </c>
-      <c r="T2" t="s">
-        <v>285</v>
-      </c>
-      <c r="U2" t="s">
-        <v>285</v>
-      </c>
-      <c r="V2">
-        <v>4</v>
-      </c>
-      <c r="W2">
-        <v>16</v>
-      </c>
-      <c r="X2" t="s">
-        <v>306</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>307</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>308</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>309</v>
-      </c>
-      <c r="AB2">
-        <v>6</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>285</v>
-      </c>
-      <c r="AD2">
-        <v>5</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>310</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>311</v>
-      </c>
-      <c r="AG2">
-        <v>0</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>311</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>311</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>311</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>311</v>
-      </c>
-      <c r="AL2">
-        <v>4</v>
-      </c>
-      <c r="AM2">
-        <v>100000</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>285</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AV2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AX2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AY2" t="s">
-        <v>312</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>312</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>312</v>
-      </c>
-      <c r="BB2" t="s">
-        <v>312</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>312</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>313</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>314</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>315</v>
-      </c>
-      <c r="BG2" t="s">
-        <v>283</v>
-      </c>
-      <c r="BH2" t="s">
-        <v>316</v>
-      </c>
-      <c r="BI2" t="s">
-        <v>283</v>
-      </c>
-      <c r="BJ2" t="s">
-        <v>285</v>
-      </c>
-      <c r="BK2" t="s">
-        <v>285</v>
-      </c>
-      <c r="BL2" t="s">
-        <v>317</v>
-      </c>
-      <c r="BM2" t="s">
-        <v>283</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>285</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>283</v>
-      </c>
-      <c r="BP2" t="s">
-        <v>285</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>283</v>
-      </c>
-      <c r="BR2" t="s">
-        <v>283</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>285</v>
-      </c>
-      <c r="BT2">
-        <v>4</v>
-      </c>
-      <c r="BU2" t="s">
-        <v>318</v>
-      </c>
-      <c r="BV2" t="s">
-        <v>283</v>
-      </c>
-      <c r="BW2" t="s">
-        <v>283</v>
-      </c>
-      <c r="BX2">
-        <v>4</v>
-      </c>
-      <c r="BY2" t="s">
-        <v>283</v>
-      </c>
-      <c r="BZ2" t="s">
-        <v>283</v>
-      </c>
-      <c r="CA2" t="s">
-        <v>283</v>
-      </c>
-      <c r="CB2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CC2" t="s">
-        <v>283</v>
-      </c>
-      <c r="CD2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CE2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CF2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CG2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CH2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CI2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CJ2">
-        <v>0</v>
-      </c>
-      <c r="CK2">
-        <v>0</v>
-      </c>
-      <c r="CL2">
-        <v>0</v>
-      </c>
-      <c r="CM2" t="s">
-        <v>283</v>
-      </c>
-      <c r="CN2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CO2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CP2" t="s">
-        <v>283</v>
-      </c>
-      <c r="CQ2" t="s">
-        <v>283</v>
-      </c>
-      <c r="CR2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CS2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CT2" t="s">
-        <v>283</v>
-      </c>
-      <c r="CU2">
-        <v>10</v>
-      </c>
-      <c r="CV2" t="s">
-        <v>283</v>
-      </c>
-      <c r="CW2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CX2" t="s">
-        <v>285</v>
-      </c>
-      <c r="CY2">
-        <v>0</v>
-      </c>
-      <c r="CZ2">
-        <v>5</v>
-      </c>
-      <c r="DA2" t="s">
-        <v>285</v>
-      </c>
-      <c r="DB2" t="s">
-        <v>283</v>
-      </c>
-      <c r="DC2" t="s">
-        <v>285</v>
-      </c>
-      <c r="DD2" t="s">
-        <v>285</v>
-      </c>
-      <c r="DE2">
-        <v>0</v>
-      </c>
-      <c r="DF2">
-        <v>0</v>
-      </c>
-      <c r="DG2">
-        <v>0</v>
-      </c>
-      <c r="DH2">
-        <v>0</v>
-      </c>
-      <c r="DI2">
-        <v>0</v>
-      </c>
-      <c r="DJ2">
-        <v>0</v>
-      </c>
-      <c r="DK2">
-        <v>0</v>
-      </c>
-      <c r="DL2">
-        <v>0</v>
-      </c>
-      <c r="DM2">
-        <v>0</v>
-      </c>
-      <c r="DN2">
-        <v>0</v>
-      </c>
-      <c r="DO2">
-        <v>0</v>
-      </c>
-      <c r="DP2">
-        <v>0</v>
-      </c>
-      <c r="DQ2">
-        <v>0</v>
-      </c>
-      <c r="DR2" t="s">
-        <v>319</v>
-      </c>
-      <c r="DS2" t="s">
-        <v>285</v>
-      </c>
-      <c r="DT2" t="s">
-        <v>283</v>
-      </c>
-      <c r="DU2">
-        <v>0</v>
-      </c>
-      <c r="DV2" t="s">
-        <v>320</v>
-      </c>
-      <c r="DW2" t="s">
-        <v>321</v>
-      </c>
-      <c r="DX2" t="s">
-        <v>285</v>
-      </c>
-      <c r="DY2" t="s">
-        <v>283</v>
-      </c>
-      <c r="DZ2" t="s">
-        <v>283</v>
-      </c>
-      <c r="EA2" t="s">
-        <v>285</v>
-      </c>
-      <c r="EB2" t="s">
-        <v>283</v>
-      </c>
-      <c r="EC2" t="s">
-        <v>285</v>
-      </c>
-      <c r="ED2" t="s">
-        <v>283</v>
-      </c>
-      <c r="EE2" t="s">
-        <v>285</v>
-      </c>
-      <c r="EF2" t="s">
-        <v>285</v>
-      </c>
-      <c r="EG2">
-        <v>0</v>
-      </c>
-      <c r="EH2">
-        <v>0</v>
-      </c>
-      <c r="EI2">
-        <v>0</v>
-      </c>
-      <c r="EJ2" t="s">
-        <v>285</v>
-      </c>
-      <c r="EK2">
-        <v>400</v>
-      </c>
-      <c r="EL2">
-        <v>53</v>
-      </c>
-      <c r="EM2">
-        <v>53</v>
-      </c>
-      <c r="EN2" t="s">
-        <v>312</v>
-      </c>
-      <c r="EO2" t="s">
-        <v>312</v>
-      </c>
-      <c r="EP2" t="s">
-        <v>312</v>
-      </c>
-      <c r="EQ2" t="s">
-        <v>312</v>
-      </c>
-      <c r="ER2" t="s">
-        <v>312</v>
-      </c>
-      <c r="ES2" t="s">
-        <v>312</v>
-      </c>
-      <c r="ET2" t="s">
-        <v>312</v>
-      </c>
-      <c r="EU2">
-        <v>0</v>
-      </c>
-      <c r="EV2">
-        <v>0</v>
-      </c>
-      <c r="EW2">
-        <v>0</v>
-      </c>
-      <c r="EX2">
-        <v>0</v>
-      </c>
-      <c r="EY2">
-        <v>0</v>
-      </c>
-      <c r="EZ2">
-        <v>0</v>
-      </c>
-      <c r="FA2">
-        <v>0</v>
-      </c>
-      <c r="FB2">
-        <v>0</v>
-      </c>
-      <c r="FC2">
-        <v>0</v>
-      </c>
-      <c r="FD2">
-        <v>0</v>
-      </c>
-      <c r="FE2">
-        <v>0</v>
-      </c>
-      <c r="FF2">
-        <v>0</v>
-      </c>
-      <c r="FG2">
-        <v>0</v>
-      </c>
-      <c r="FH2">
-        <v>0</v>
-      </c>
-      <c r="FI2">
-        <v>0</v>
-      </c>
-      <c r="FJ2">
-        <v>0</v>
-      </c>
-      <c r="FK2">
-        <v>0</v>
-      </c>
-      <c r="FL2">
-        <v>0</v>
-      </c>
-      <c r="FM2">
-        <v>0</v>
-      </c>
-      <c r="FN2">
-        <v>0</v>
-      </c>
-      <c r="FO2">
-        <v>0</v>
-      </c>
-      <c r="FP2">
-        <v>0</v>
-      </c>
-      <c r="FQ2">
-        <v>0</v>
-      </c>
-      <c r="FR2">
-        <v>0</v>
-      </c>
-      <c r="FS2">
-        <v>0</v>
-      </c>
-      <c r="FT2">
-        <v>0</v>
-      </c>
-      <c r="FU2">
-        <v>0</v>
-      </c>
-      <c r="FV2" t="s">
-        <v>302</v>
-      </c>
-      <c r="FW2" t="s">
-        <v>303</v>
-      </c>
-      <c r="FX2" t="s">
-        <v>304</v>
-      </c>
-      <c r="FY2">
-        <v>115</v>
-      </c>
-      <c r="FZ2">
-        <v>0</v>
-      </c>
-      <c r="GA2">
-        <v>0</v>
-      </c>
-      <c r="GB2">
-        <v>0</v>
-      </c>
-      <c r="GC2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:185" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>293</v>
       </c>
       <c r="B3" t="s">
         <v>291</v>
@@ -2684,10 +2741,10 @@
         <v>345</v>
       </c>
       <c r="D3" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E3" t="s">
-        <v>322</v>
+        <v>299</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>301</v>
@@ -2714,10 +2771,10 @@
         <v>2600</v>
       </c>
       <c r="N3">
-        <v>1350</v>
+        <v>1390</v>
       </c>
       <c r="O3">
-        <v>11.739130434782609</v>
+        <v>12.086956521739131</v>
       </c>
       <c r="P3" t="s">
         <v>305</v>
@@ -2753,10 +2810,10 @@
         <v>308</v>
       </c>
       <c r="AA3" t="s">
-        <v>323</v>
+        <v>309</v>
       </c>
       <c r="AB3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC3" t="s">
         <v>285</v>
@@ -2882,10 +2939,10 @@
         <v>283</v>
       </c>
       <c r="BR3" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="BS3" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="BT3">
         <v>4</v>
@@ -2903,7 +2960,7 @@
         <v>4</v>
       </c>
       <c r="BY3" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="BZ3" t="s">
         <v>283</v>
@@ -3053,7 +3110,7 @@
         <v>320</v>
       </c>
       <c r="DW3" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="DX3" t="s">
         <v>285</v>
@@ -3211,11 +3268,11 @@
       <c r="FW3" t="s">
         <v>303</v>
       </c>
-      <c r="FX3" t="s">
-        <v>304</v>
+      <c r="FX3">
+        <v>115</v>
       </c>
       <c r="FY3">
-        <v>115</v>
+        <v>0</v>
       </c>
       <c r="FZ3">
         <v>0</v>
@@ -3227,12 +3284,24 @@
         <v>0</v>
       </c>
       <c r="GC3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:185" x14ac:dyDescent="0.3">
+        <v>1598</v>
+      </c>
+      <c r="GD3" t="s">
+        <v>356</v>
+      </c>
+      <c r="GE3" t="s">
+        <v>357</v>
+      </c>
+      <c r="GF3" t="s">
+        <v>358</v>
+      </c>
+      <c r="GG3" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="4" spans="1:189" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B4" t="s">
         <v>291</v>
@@ -3241,13 +3310,13 @@
         <v>345</v>
       </c>
       <c r="D4" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E4" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>326</v>
+        <v>301</v>
       </c>
       <c r="G4" t="s">
         <v>304</v>
@@ -3259,31 +3328,31 @@
         <v>0</v>
       </c>
       <c r="J4">
-        <v>4500</v>
+        <v>4335</v>
       </c>
       <c r="K4">
-        <v>1855</v>
+        <v>1825</v>
       </c>
       <c r="L4">
-        <v>1690</v>
+        <v>1660</v>
       </c>
       <c r="M4">
-        <v>2650</v>
+        <v>2600</v>
       </c>
       <c r="N4">
-        <v>1535</v>
+        <v>1350</v>
       </c>
       <c r="O4">
-        <v>9.9032258064516121</v>
+        <v>11.739130434782609</v>
       </c>
       <c r="P4" t="s">
-        <v>327</v>
+        <v>305</v>
       </c>
       <c r="Q4" t="s">
         <v>283</v>
       </c>
       <c r="R4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S4" t="s">
         <v>283</v>
@@ -3301,7 +3370,7 @@
         <v>16</v>
       </c>
       <c r="X4" t="s">
-        <v>328</v>
+        <v>306</v>
       </c>
       <c r="Y4" t="s">
         <v>307</v>
@@ -3310,10 +3379,10 @@
         <v>308</v>
       </c>
       <c r="AA4" t="s">
-        <v>309</v>
+        <v>323</v>
       </c>
       <c r="AB4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AC4" t="s">
         <v>285</v>
@@ -3418,7 +3487,7 @@
         <v>285</v>
       </c>
       <c r="BK4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="BL4" t="s">
         <v>317</v>
@@ -3439,13 +3508,13 @@
         <v>283</v>
       </c>
       <c r="BR4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="BS4" t="s">
         <v>283</v>
       </c>
       <c r="BT4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BU4" t="s">
         <v>318</v>
@@ -3460,7 +3529,7 @@
         <v>4</v>
       </c>
       <c r="BY4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="BZ4" t="s">
         <v>283</v>
@@ -3478,7 +3547,7 @@
         <v>285</v>
       </c>
       <c r="CE4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="CF4" t="s">
         <v>285</v>
@@ -3508,7 +3577,7 @@
         <v>285</v>
       </c>
       <c r="CO4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="CP4" t="s">
         <v>283</v>
@@ -3526,7 +3595,7 @@
         <v>283</v>
       </c>
       <c r="CU4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="CV4" t="s">
         <v>283</v>
@@ -3598,7 +3667,7 @@
         <v>319</v>
       </c>
       <c r="DS4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="DT4" t="s">
         <v>283</v>
@@ -3607,10 +3676,10 @@
         <v>0</v>
       </c>
       <c r="DV4" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
       <c r="DW4" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="DX4" t="s">
         <v>285</v>
@@ -3619,19 +3688,19 @@
         <v>283</v>
       </c>
       <c r="DZ4" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="EA4" t="s">
+        <v>285</v>
+      </c>
+      <c r="EB4" t="s">
         <v>283</v>
       </c>
-      <c r="EB4" t="s">
-        <v>285</v>
-      </c>
       <c r="EC4" t="s">
         <v>285</v>
       </c>
       <c r="ED4" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="EE4" t="s">
         <v>285</v>
@@ -3652,13 +3721,13 @@
         <v>285</v>
       </c>
       <c r="EK4">
-        <v>475</v>
+        <v>400</v>
       </c>
       <c r="EL4">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="EM4">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="EN4" t="s">
         <v>312</v>
@@ -3768,31 +3837,612 @@
       <c r="FW4" t="s">
         <v>303</v>
       </c>
-      <c r="FX4" t="s">
+      <c r="FX4">
+        <v>115</v>
+      </c>
+      <c r="FY4">
+        <v>0</v>
+      </c>
+      <c r="FZ4">
+        <v>0</v>
+      </c>
+      <c r="GA4">
+        <v>0</v>
+      </c>
+      <c r="GB4">
+        <v>0</v>
+      </c>
+      <c r="GC4">
+        <v>1598</v>
+      </c>
+      <c r="GD4" t="s">
+        <v>356</v>
+      </c>
+      <c r="GE4" t="s">
+        <v>312</v>
+      </c>
+      <c r="GF4" t="s">
+        <v>358</v>
+      </c>
+      <c r="GG4" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="5" spans="1:189" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>294</v>
+      </c>
+      <c r="B5" t="s">
+        <v>291</v>
+      </c>
+      <c r="C5" t="s">
+        <v>345</v>
+      </c>
+      <c r="D5" t="s">
+        <v>348</v>
+      </c>
+      <c r="E5" t="s">
+        <v>325</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="G5" t="s">
         <v>304</v>
       </c>
-      <c r="FY4">
+      <c r="H5" t="s">
+        <v>300</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>4500</v>
+      </c>
+      <c r="K5">
+        <v>1855</v>
+      </c>
+      <c r="L5">
+        <v>1690</v>
+      </c>
+      <c r="M5">
+        <v>2650</v>
+      </c>
+      <c r="N5">
+        <v>1535</v>
+      </c>
+      <c r="O5">
+        <v>9.9032258064516121</v>
+      </c>
+      <c r="P5" t="s">
+        <v>327</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>283</v>
+      </c>
+      <c r="R5">
+        <v>18</v>
+      </c>
+      <c r="S5" t="s">
+        <v>283</v>
+      </c>
+      <c r="T5" t="s">
+        <v>285</v>
+      </c>
+      <c r="U5" t="s">
+        <v>285</v>
+      </c>
+      <c r="V5">
+        <v>4</v>
+      </c>
+      <c r="W5">
+        <v>16</v>
+      </c>
+      <c r="X5" t="s">
+        <v>328</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>307</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>308</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>309</v>
+      </c>
+      <c r="AB5">
+        <v>6</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>285</v>
+      </c>
+      <c r="AD5">
+        <v>5</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>310</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>311</v>
+      </c>
+      <c r="AG5">
+        <v>0</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>311</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>311</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>311</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>311</v>
+      </c>
+      <c r="AL5">
+        <v>4</v>
+      </c>
+      <c r="AM5">
+        <v>100000</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>285</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AS5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AT5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AU5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AV5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AX5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AY5" t="s">
+        <v>312</v>
+      </c>
+      <c r="AZ5" t="s">
+        <v>312</v>
+      </c>
+      <c r="BA5" t="s">
+        <v>312</v>
+      </c>
+      <c r="BB5" t="s">
+        <v>312</v>
+      </c>
+      <c r="BC5" t="s">
+        <v>312</v>
+      </c>
+      <c r="BD5" t="s">
+        <v>313</v>
+      </c>
+      <c r="BE5" t="s">
+        <v>314</v>
+      </c>
+      <c r="BF5" t="s">
+        <v>315</v>
+      </c>
+      <c r="BG5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BH5" t="s">
+        <v>316</v>
+      </c>
+      <c r="BI5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BJ5" t="s">
+        <v>285</v>
+      </c>
+      <c r="BK5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BL5" t="s">
+        <v>317</v>
+      </c>
+      <c r="BM5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BN5" t="s">
+        <v>285</v>
+      </c>
+      <c r="BO5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BP5" t="s">
+        <v>285</v>
+      </c>
+      <c r="BQ5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BR5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BS5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BT5">
+        <v>6</v>
+      </c>
+      <c r="BU5" t="s">
+        <v>318</v>
+      </c>
+      <c r="BV5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BW5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BX5">
+        <v>4</v>
+      </c>
+      <c r="BY5" t="s">
+        <v>283</v>
+      </c>
+      <c r="BZ5" t="s">
+        <v>283</v>
+      </c>
+      <c r="CA5" t="s">
+        <v>283</v>
+      </c>
+      <c r="CB5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CC5" t="s">
+        <v>283</v>
+      </c>
+      <c r="CD5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CE5" t="s">
+        <v>283</v>
+      </c>
+      <c r="CF5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CG5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CH5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CI5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CJ5">
+        <v>0</v>
+      </c>
+      <c r="CK5">
+        <v>0</v>
+      </c>
+      <c r="CL5">
+        <v>0</v>
+      </c>
+      <c r="CM5" t="s">
+        <v>283</v>
+      </c>
+      <c r="CN5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CO5" t="s">
+        <v>283</v>
+      </c>
+      <c r="CP5" t="s">
+        <v>283</v>
+      </c>
+      <c r="CQ5" t="s">
+        <v>283</v>
+      </c>
+      <c r="CR5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CS5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CT5" t="s">
+        <v>283</v>
+      </c>
+      <c r="CU5">
+        <v>9</v>
+      </c>
+      <c r="CV5" t="s">
+        <v>283</v>
+      </c>
+      <c r="CW5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CX5" t="s">
+        <v>285</v>
+      </c>
+      <c r="CY5">
+        <v>0</v>
+      </c>
+      <c r="CZ5">
+        <v>5</v>
+      </c>
+      <c r="DA5" t="s">
+        <v>285</v>
+      </c>
+      <c r="DB5" t="s">
+        <v>283</v>
+      </c>
+      <c r="DC5" t="s">
+        <v>285</v>
+      </c>
+      <c r="DD5" t="s">
+        <v>285</v>
+      </c>
+      <c r="DE5">
+        <v>0</v>
+      </c>
+      <c r="DF5">
+        <v>0</v>
+      </c>
+      <c r="DG5">
+        <v>0</v>
+      </c>
+      <c r="DH5">
+        <v>0</v>
+      </c>
+      <c r="DI5">
+        <v>0</v>
+      </c>
+      <c r="DJ5">
+        <v>0</v>
+      </c>
+      <c r="DK5">
+        <v>0</v>
+      </c>
+      <c r="DL5">
+        <v>0</v>
+      </c>
+      <c r="DM5">
+        <v>0</v>
+      </c>
+      <c r="DN5">
+        <v>0</v>
+      </c>
+      <c r="DO5">
+        <v>0</v>
+      </c>
+      <c r="DP5">
+        <v>0</v>
+      </c>
+      <c r="DQ5">
+        <v>0</v>
+      </c>
+      <c r="DR5" t="s">
+        <v>319</v>
+      </c>
+      <c r="DS5" t="s">
+        <v>283</v>
+      </c>
+      <c r="DT5" t="s">
+        <v>283</v>
+      </c>
+      <c r="DU5">
+        <v>0</v>
+      </c>
+      <c r="DV5" t="s">
+        <v>329</v>
+      </c>
+      <c r="DW5" t="s">
+        <v>330</v>
+      </c>
+      <c r="DX5" t="s">
+        <v>285</v>
+      </c>
+      <c r="DY5" t="s">
+        <v>283</v>
+      </c>
+      <c r="DZ5" t="s">
+        <v>285</v>
+      </c>
+      <c r="EA5" t="s">
+        <v>283</v>
+      </c>
+      <c r="EB5" t="s">
+        <v>285</v>
+      </c>
+      <c r="EC5" t="s">
+        <v>285</v>
+      </c>
+      <c r="ED5" t="s">
+        <v>285</v>
+      </c>
+      <c r="EE5" t="s">
+        <v>285</v>
+      </c>
+      <c r="EF5" t="s">
+        <v>285</v>
+      </c>
+      <c r="EG5">
+        <v>0</v>
+      </c>
+      <c r="EH5">
+        <v>0</v>
+      </c>
+      <c r="EI5">
+        <v>0</v>
+      </c>
+      <c r="EJ5" t="s">
+        <v>285</v>
+      </c>
+      <c r="EK5">
+        <v>475</v>
+      </c>
+      <c r="EL5">
+        <v>58</v>
+      </c>
+      <c r="EM5">
+        <v>58</v>
+      </c>
+      <c r="EN5" t="s">
+        <v>312</v>
+      </c>
+      <c r="EO5" t="s">
+        <v>312</v>
+      </c>
+      <c r="EP5" t="s">
+        <v>312</v>
+      </c>
+      <c r="EQ5" t="s">
+        <v>312</v>
+      </c>
+      <c r="ER5" t="s">
+        <v>312</v>
+      </c>
+      <c r="ES5" t="s">
+        <v>312</v>
+      </c>
+      <c r="ET5" t="s">
+        <v>312</v>
+      </c>
+      <c r="EU5">
+        <v>0</v>
+      </c>
+      <c r="EV5">
+        <v>0</v>
+      </c>
+      <c r="EW5">
+        <v>0</v>
+      </c>
+      <c r="EX5">
+        <v>0</v>
+      </c>
+      <c r="EY5">
+        <v>0</v>
+      </c>
+      <c r="EZ5">
+        <v>0</v>
+      </c>
+      <c r="FA5">
+        <v>0</v>
+      </c>
+      <c r="FB5">
+        <v>0</v>
+      </c>
+      <c r="FC5">
+        <v>0</v>
+      </c>
+      <c r="FD5">
+        <v>0</v>
+      </c>
+      <c r="FE5">
+        <v>0</v>
+      </c>
+      <c r="FF5">
+        <v>0</v>
+      </c>
+      <c r="FG5">
+        <v>0</v>
+      </c>
+      <c r="FH5">
+        <v>0</v>
+      </c>
+      <c r="FI5">
+        <v>0</v>
+      </c>
+      <c r="FJ5">
+        <v>0</v>
+      </c>
+      <c r="FK5">
+        <v>0</v>
+      </c>
+      <c r="FL5">
+        <v>0</v>
+      </c>
+      <c r="FM5">
+        <v>0</v>
+      </c>
+      <c r="FN5">
+        <v>0</v>
+      </c>
+      <c r="FO5">
+        <v>0</v>
+      </c>
+      <c r="FP5">
+        <v>0</v>
+      </c>
+      <c r="FQ5">
+        <v>0</v>
+      </c>
+      <c r="FR5">
+        <v>0</v>
+      </c>
+      <c r="FS5">
+        <v>0</v>
+      </c>
+      <c r="FT5">
+        <v>0</v>
+      </c>
+      <c r="FU5">
+        <v>0</v>
+      </c>
+      <c r="FV5" t="s">
+        <v>302</v>
+      </c>
+      <c r="FW5" t="s">
+        <v>303</v>
+      </c>
+      <c r="FX5">
         <v>155</v>
       </c>
-      <c r="FZ4">
-        <v>0</v>
-      </c>
-      <c r="GA4">
-        <v>0</v>
-      </c>
-      <c r="GB4">
-        <v>0</v>
-      </c>
-      <c r="GC4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:185" x14ac:dyDescent="0.3">
+      <c r="FY5">
+        <v>0</v>
+      </c>
+      <c r="FZ5">
+        <v>0</v>
+      </c>
+      <c r="GA5">
+        <v>0</v>
+      </c>
+      <c r="GB5">
+        <v>0</v>
+      </c>
+      <c r="GC5">
+        <v>1499</v>
+      </c>
+      <c r="GD5" t="s">
+        <v>356</v>
+      </c>
+      <c r="GE5" t="s">
+        <v>360</v>
+      </c>
+      <c r="GF5" t="s">
+        <v>358</v>
+      </c>
+      <c r="GG5" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="8" spans="1:189" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="11" spans="1:185" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:189" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>295</v>
       </c>
@@ -3806,7 +4456,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="12" spans="1:185" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:189" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>350</v>
       </c>

</xml_diff>